<commit_message>
Update Himaja postcode pin
</commit_message>
<xml_diff>
--- a/Skipton - CGI partners travel.xlsx
+++ b/Skipton - CGI partners travel.xlsx
@@ -706,7 +706,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -768,7 +768,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -806,7 +806,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -1021,7 +1021,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -1144,7 +1144,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1206,7 +1206,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -3573,7 +3573,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>M50</t>
+          <t>M33 7GG</t>
         </is>
       </c>
       <c r="D21" s="36" t="n">
@@ -5796,8 +5796,8 @@
     <col width="28.33203125" bestFit="1" customWidth="1" style="5" min="2" max="2"/>
     <col width="17.33203125" bestFit="1" customWidth="1" style="5" min="3" max="6"/>
     <col width="11" bestFit="1" customWidth="1" style="5" min="7" max="8"/>
-    <col width="8.83203125" customWidth="1" style="5" min="9" max="9"/>
-    <col width="8.83203125" customWidth="1" style="5" min="10" max="16384"/>
+    <col width="8.83203125" customWidth="1" style="5" min="9" max="10"/>
+    <col width="8.83203125" customWidth="1" style="5" min="11" max="16384"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -7479,8 +7479,8 @@
     <col width="36" bestFit="1" customWidth="1" style="5" min="6" max="7"/>
     <col width="40.5" bestFit="1" customWidth="1" style="5" min="8" max="8"/>
     <col width="19.83203125" bestFit="1" customWidth="1" style="5" min="9" max="9"/>
-    <col width="8.83203125" customWidth="1" style="5" min="10" max="10"/>
-    <col width="8.83203125" customWidth="1" style="5" min="11" max="16384"/>
+    <col width="8.83203125" customWidth="1" style="5" min="10" max="11"/>
+    <col width="8.83203125" customWidth="1" style="5" min="12" max="16384"/>
   </cols>
   <sheetData>
     <row r="3" ht="16" customHeight="1">
@@ -7835,8 +7835,8 @@
     <col width="16.83203125" bestFit="1" customWidth="1" style="5" min="2" max="4"/>
     <col width="10.5" bestFit="1" customWidth="1" style="5" min="5" max="7"/>
     <col width="11" bestFit="1" customWidth="1" style="5" min="8" max="8"/>
-    <col width="8.83203125" customWidth="1" style="5" min="9" max="9"/>
-    <col width="8.83203125" customWidth="1" style="5" min="10" max="16384"/>
+    <col width="8.83203125" customWidth="1" style="5" min="9" max="10"/>
+    <col width="8.83203125" customWidth="1" style="5" min="11" max="16384"/>
   </cols>
   <sheetData>
     <row r="3" ht="16" customHeight="1">
@@ -8534,8 +8534,8 @@
   <dimension ref="A1:AH373"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="8.83203125" customWidth="1" style="5" min="1" max="1"/>
-    <col width="8.83203125" customWidth="1" style="5" min="2" max="16384"/>
+    <col width="8.83203125" customWidth="1" style="5" min="1" max="2"/>
+    <col width="8.83203125" customWidth="1" style="5" min="3" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add Paresh postcode pin
</commit_message>
<xml_diff>
--- a/Skipton - CGI partners travel.xlsx
+++ b/Skipton - CGI partners travel.xlsx
@@ -706,7 +706,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -768,7 +768,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -806,7 +806,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -1021,7 +1021,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -1144,7 +1144,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1206,7 +1206,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -4230,9 +4230,22 @@
           <t>Paresh Rathod</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>LS16 6JN</t>
+        </is>
+      </c>
+      <c r="D43" s="36" t="n">
+        <v>2</v>
+      </c>
       <c r="E43" t="inlineStr">
         <is>
           <t>Romy</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>3 days per week</t>
         </is>
       </c>
     </row>
@@ -5796,8 +5809,8 @@
     <col width="28.33203125" bestFit="1" customWidth="1" style="5" min="2" max="2"/>
     <col width="17.33203125" bestFit="1" customWidth="1" style="5" min="3" max="6"/>
     <col width="11" bestFit="1" customWidth="1" style="5" min="7" max="8"/>
-    <col width="8.83203125" customWidth="1" style="5" min="9" max="10"/>
-    <col width="8.83203125" customWidth="1" style="5" min="11" max="16384"/>
+    <col width="8.83203125" customWidth="1" style="5" min="9" max="11"/>
+    <col width="8.83203125" customWidth="1" style="5" min="12" max="16384"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -7479,8 +7492,8 @@
     <col width="36" bestFit="1" customWidth="1" style="5" min="6" max="7"/>
     <col width="40.5" bestFit="1" customWidth="1" style="5" min="8" max="8"/>
     <col width="19.83203125" bestFit="1" customWidth="1" style="5" min="9" max="9"/>
-    <col width="8.83203125" customWidth="1" style="5" min="10" max="11"/>
-    <col width="8.83203125" customWidth="1" style="5" min="12" max="16384"/>
+    <col width="8.83203125" customWidth="1" style="5" min="10" max="12"/>
+    <col width="8.83203125" customWidth="1" style="5" min="13" max="16384"/>
   </cols>
   <sheetData>
     <row r="3" ht="16" customHeight="1">
@@ -7835,8 +7848,8 @@
     <col width="16.83203125" bestFit="1" customWidth="1" style="5" min="2" max="4"/>
     <col width="10.5" bestFit="1" customWidth="1" style="5" min="5" max="7"/>
     <col width="11" bestFit="1" customWidth="1" style="5" min="8" max="8"/>
-    <col width="8.83203125" customWidth="1" style="5" min="9" max="10"/>
-    <col width="8.83203125" customWidth="1" style="5" min="11" max="16384"/>
+    <col width="8.83203125" customWidth="1" style="5" min="9" max="11"/>
+    <col width="8.83203125" customWidth="1" style="5" min="12" max="16384"/>
   </cols>
   <sheetData>
     <row r="3" ht="16" customHeight="1">
@@ -8534,8 +8547,8 @@
   <dimension ref="A1:AH373"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="8.83203125" customWidth="1" style="5" min="1" max="2"/>
-    <col width="8.83203125" customWidth="1" style="5" min="3" max="16384"/>
+    <col width="8.83203125" customWidth="1" style="5" min="1" max="3"/>
+    <col width="8.83203125" customWidth="1" style="5" min="4" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>